<commit_message>
Demo IWP 3.0 & Online Reporting Search Results Test cases
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPCCData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPCCData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="141">
   <si>
     <t>Result</t>
   </si>
@@ -472,6 +472,12 @@
   </si>
   <si>
     <t>Tue Jun 09 01:32:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Aug 19 22:01:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Aug 19 22:04:07 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -809,7 +815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A8F394B-F089-4FB3-82A1-125786B1E619}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -895,7 +901,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE94437-153A-41B2-A46E-2F45E61989DF}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -943,11 +949,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
-        <v>136</v>
+      <c r="B2" t="s" s="0">
+        <v>140</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -987,7 +993,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{093A05D5-CD46-4FC8-83C2-DE55EC3B00E1}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1035,10 +1041,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>130</v>
       </c>
       <c r="C2" s="2"/>
@@ -1079,7 +1085,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A6F3014-83EE-40CF-BEA6-9E7A762354AA}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1127,10 +1133,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>125</v>
       </c>
       <c r="C2" s="2"/>
@@ -1171,7 +1177,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{434CAF96-FDCD-425D-B74E-26C08061546A}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1219,10 +1225,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>126</v>
       </c>
       <c r="C2" s="2"/>
@@ -1263,7 +1269,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87175E7B-348C-48F8-975E-573E1AA57C35}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1311,10 +1317,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>32</v>
       </c>
       <c r="C2" s="2"/>
@@ -1355,7 +1361,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF76F2B3-5F15-409A-AC34-86B0DD8FC5F1}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1403,10 +1409,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>127</v>
       </c>
       <c r="C2" s="2"/>
@@ -1447,7 +1453,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF1CC49-076D-4B64-8F44-11F5FA5C3B7C}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1495,10 +1501,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>128</v>
       </c>
       <c r="C2" s="2"/>
@@ -1539,7 +1545,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A016DD-A4BF-47A4-99DE-0B94685F9A61}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1587,10 +1593,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>129</v>
       </c>
       <c r="C2" s="2"/>
@@ -1631,7 +1637,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D4D6FED-07DF-4BD9-BB91-007F4EF89576}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1679,10 +1685,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>131</v>
       </c>
       <c r="C2" s="2"/>
@@ -1723,7 +1729,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE865A-189F-47E2-B372-099EB34B0721}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1771,10 +1777,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>132</v>
       </c>
       <c r="C2" s="2"/>
@@ -1815,7 +1821,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6E76688-C590-48CE-8843-48B79B2A30B7}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1901,7 +1907,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B29E0A75-769C-43A6-A3D3-703A1A1AFA44}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1949,10 +1955,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>133</v>
       </c>
       <c r="C2" s="2"/>
@@ -1993,7 +1999,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2041,11 +2047,11 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
-        <v>135</v>
+      <c r="B2" t="s" s="0">
+        <v>139</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2088,7 +2094,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B2AA229-8633-483E-A009-0064BA327142}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" customWidth="true" width="27.77734375" collapsed="true"/>
@@ -2139,10 +2145,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>137</v>
       </c>
       <c r="C2" s="2"/>
@@ -2185,7 +2191,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E49D1CA0-9ECE-4C77-A64C-43CA3156CCD7}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2271,7 +2277,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF4DDCDE-4C11-464F-9492-FC8FE5D5A265}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2319,10 +2325,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>123</v>
       </c>
       <c r="C2" s="2"/>
@@ -2363,7 +2369,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61EC5E6A-6755-4451-A097-7A8CEE1F522B}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2411,10 +2417,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>124</v>
       </c>
       <c r="C2" s="2"/>
@@ -2455,7 +2461,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46BFFB65-1565-4A34-B0E7-464EF87C75A7}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2503,10 +2509,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>138</v>
       </c>
       <c r="C2" s="2"/>
@@ -2547,7 +2553,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125BE3DD-7AC0-404A-8C39-EB8ECFFFBDDD}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -2595,10 +2601,10 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>134</v>
       </c>
       <c r="C2" s="2"/>

</xml_diff>